<commit_message>
Updated some of the recommendations, added two additional test files - one with comment lines, the other with no %
</commit_message>
<xml_diff>
--- a/dash-config-sim.xlsx
+++ b/dash-config-sim.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Technical\Utilities\Python\dash-lineplot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1576989-6E46-4C4D-8DBC-1447BC9D989E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479F9DDF-FC26-43F8-B35C-4736781C8F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="-15405" windowWidth="18690" windowHeight="14235" tabRatio="686" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="22920" windowHeight="14115" tabRatio="686" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="header" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="149">
   <si>
     <t>Variable</t>
   </si>
@@ -470,9 +470,6 @@
     <t>min</t>
   </si>
   <si>
-    <t>std</t>
-  </si>
-  <si>
     <t>frTime[s]</t>
   </si>
   <si>
@@ -488,7 +485,16 @@
     <t>z [m]</t>
   </si>
   <si>
-    <t>data/sensor-tel.txt</t>
+    <t>data/sensor-tel-test1.txt</t>
+  </si>
+  <si>
+    <t>data/sensor-tel-test2.txt</t>
+  </si>
+  <si>
+    <t>stdx10</t>
+  </si>
+  <si>
+    <t>data/sensor-tel-test3.txt</t>
   </si>
 </sst>
 </file>
@@ -994,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.1328125" customWidth="1"/>
@@ -1064,7 +1070,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1102,7 +1108,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -1194,7 +1200,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -1212,7 +1218,7 @@
         <v>18</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>74</v>
@@ -1232,7 +1238,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
@@ -1266,7 +1272,15 @@
         <v>86</v>
       </c>
       <c r="B15" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A16" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="15" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1346,7 +1360,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1384,7 +1398,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -1420,7 +1434,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1438,7 +1452,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>74</v>
@@ -1458,7 +1472,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="4"/>
@@ -1489,7 +1503,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B12" s="15" t="b">
         <v>0</v>
@@ -1571,7 +1585,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1607,7 +1621,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -1699,7 +1713,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
@@ -1719,7 +1733,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
@@ -1752,7 +1766,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B14" s="15" t="b">
         <v>0</v>
@@ -1870,7 +1884,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2019,7 +2033,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B14" s="15" t="b">
         <v>0</v>
@@ -2138,7 +2152,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2254,7 +2268,7 @@
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4">
@@ -2285,7 +2299,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B14" s="15" t="b">
         <v>0</v>
@@ -9797,7 +9811,7 @@
       </c>
     </row>
     <row r="54" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="55" spans="1:2" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:2" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A55" s="11" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
added legend display parameters rewrote all docs
</commit_message>
<xml_diff>
--- a/dash-config-sim.xlsx
+++ b/dash-config-sim.xlsx
@@ -937,7 +937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.86328125" style="13" customWidth="1"/>
@@ -990,6 +990,16 @@
       </c>
       <c r="B6" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LegendTransparency</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2322,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:AMK85"/>
+  <dimension ref="A1:AMK92"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.6640625" style="11" customWidth="1"/>
@@ -9989,6 +9999,85 @@
         <v>125</v>
       </c>
     </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Changed 2026-10-08:</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LegendTransparency</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number from 0 to 1: transparency of the legend's white background, 0 solid white, 1 fully see-through (the plot shows); default 0.4. In the header it sets the whole page; a row before a sheet's first Title sets that tab; a row after a graph's Title (before the next Title) sets that graph only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HardcopyGraphsPerPage</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive whole number: equal-height graph slots per hardcopy page (Ctrl+Alt+H) for this tab. Without it, graphs keep their on-screen heights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">xValue (column)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On a yValue row: the x column for that line only, looked up in its own Datafile, for files that name their time column differently. The x scale, offset and label stay the block's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LegendOrientation</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'v' (default) or 'h': the legend's entries in a column or a row. Same three levels as LegendTransparency: header, sheet row before the first Title, row after a graph's Title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LegendX</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number from 0 to 1 (default 1): the legend position across the plot area, 0 left edge, 1 right edge. The legend anchors on its nearest side. Same three levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LegendY</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number from 0 to 1 (default 1): the legend position up the plot area, 0 bottom, 1 top. Kept inside 0..1 so stacked graphs stay aligned in x. Same three levels.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A9:B9"/>

</xml_diff>